<commit_message>
Update train driver research with live vacancy checks
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RsSQ2cbMw8nQp1fJSBRRWh
</commit_message>
<xml_diff>
--- a/train_driver_research/london_train_driver_apprenticeships.xlsx
+++ b/train_driver_research/london_train_driver_apprenticeships.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Sources" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Operators'!$A$1:$N$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Operators'!$A$1:$N$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -888,6 +888,18 @@
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>4 Oct 2026 live check: the government Find an Apprenticeship service shows 0 train driver apprenticeships within 40 miles of London, and SWR and Elizabeth line (GTS) list no open driver vacancies – only talent pools. Several operators (TfL, East Midlands, London Northwestern, railforums) sit behind Cloudflare bot protection and could not be read; I did not try to bypass it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>5.</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Rail ownership is in flux (government is moving operators into public ownership / Great British Railways), so company names and recruitment arrangements are changing – e.g. the Elizabeth line is now run by GTS Rail Operations.</t>
         </is>
@@ -904,7 +916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1019,7 +1031,7 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>£27,639 start → £33,867 after Rules &amp; Regs (~3 mths) → £54,002 on completing apprenticeship (~12 mths) → £62,727 after 12 mths qualified. 28 days leave, final-salary pension, free travel.</t>
+          <t>£27,639 start → £33,867 after Rules &amp; Regs (~3 mths) → £54,002 on completing apprenticeship (~12 mths) → £62,727 after 12 mths qualified. 28 days leave, final-salary pension, free travel. (2024 round: £33,510 → £68,958 – older pay scale.)</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
@@ -1112,7 +1124,7 @@
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Closed 19 Jun 2026 (15 posts). Rolling windows – check careers.gtsr.co.uk</t>
+          <t>Closed 19 Jun 2026 (15 posts). Checked 4 Oct 2026: 0 driver vacancies, but a 'Trainee train driver' talent pool is open to register on careers.gtsr.co.uk</t>
         </is>
       </c>
       <c r="L3" s="9" t="inlineStr">
@@ -1127,7 +1139,7 @@
       </c>
       <c r="N3" s="7" t="inlineStr">
         <is>
-          <t>Seen via job-listing aggregation, not the official page</t>
+          <t>Salary from job-listing aggregation; official careers site read 4 Oct 2026 (status only, no salary shown)</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1326,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Rolling – check careers.southwesternrailway.com</t>
+          <t>Checked 4 Oct 2026: no trainee driver vacancies listed – register for alerts</t>
         </is>
       </c>
       <c r="L6" s="9" t="inlineStr">
@@ -1329,7 +1341,7 @@
       </c>
       <c r="N6" s="7" t="inlineStr">
         <is>
-          <t>Search result from SWR adverts; page itself had no detail</t>
+          <t>Salary from earlier SWR adverts; careers site read 4 Oct 2026 (no live driver roles)</t>
         </is>
       </c>
     </row>
@@ -1668,24 +1680,24 @@
     <row r="12" ht="110" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>First Rail London (ex-Arriva Rail London)</t>
+          <t>Avanti West Coast</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Trainee Train Driver</t>
+          <t>Trainee Train Driver – Euston talent pool</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>London (took over concession 2 May 2026)</t>
+          <t>London Euston</t>
         </is>
       </c>
       <c r="D12" s="7" t="n"/>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>No salary found.</t>
+          <t>Listed as a talent pool on railwaycareers.co.uk; no salary shown (sector range quoted £27k–£33k).</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1710,12 +1722,12 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>A window closed on a 23rd in May 2026 – details unconfirmed</t>
+          <t>Talent pool listed – register interest on Avanti careers site</t>
         </is>
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>https://careers.firstgroup.co.uk/</t>
+          <t>https://www.avantiwestcoast.co.uk/careers</t>
         </is>
       </c>
       <c r="M12" s="12" t="inlineStr">
@@ -1725,63 +1737,61 @@
       </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
-          <t>Forum mention only</t>
+          <t>Aggregator listing only</t>
         </is>
       </c>
     </row>
     <row r="13" ht="110" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Greater Anglia</t>
+          <t>First Rail London (ex-Arriva Rail London)</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Trainee Mainline Driver</t>
+          <t>Trainee Train Driver</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>London Liverpool Street</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>25120</v>
-      </c>
+          <t>London (took over concession 2 May 2026)</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n"/>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>£25,120 is from an EXPIRED older posting – likely out of date.</t>
+          <t>No salary found.</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>~18 months</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>21 (for qualified post)</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>Not confirmed</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Near depot</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>Currently advertising conductors (closed 7 Aug 2026) – drivers not confirmed</t>
+          <t>A window closed on a 23rd in May 2026 – details unconfirmed</t>
         </is>
       </c>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t>https://apply.greateranglia.co.uk/</t>
+          <t>https://careers.firstgroup.co.uk/</t>
         </is>
       </c>
       <c r="M13" s="12" t="inlineStr">
@@ -1791,45 +1801,43 @@
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>Old posting</t>
+          <t>Forum mention only</t>
         </is>
       </c>
     </row>
     <row r="14" ht="110" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>DB Cargo (freight)</t>
+          <t>Greater Anglia</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Junior Train Driver</t>
+          <t>Trainee Mainline Driver</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Not London-specific (national depots)</t>
+          <t>London Liverpool Street</t>
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>31381</v>
-      </c>
-      <c r="E14" s="8" t="n">
-        <v>55525</v>
-      </c>
+        <v>25120</v>
+      </c>
+      <c r="E14" s="7" t="n"/>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>£31,381 start → £55,525 qualified.</t>
+          <t>£25,120 is from an EXPIRED older posting – likely out of date.</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>~12–18 months</t>
+          <t>~18 months</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Check advert</t>
+          <t>21 (for qualified post)</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
@@ -1839,17 +1847,17 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>Depot dependent</t>
+          <t>Near depot</t>
         </is>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>Talent-pool style</t>
+          <t>Currently advertising conductors (closed 7 Aug 2026) – drivers not confirmed</t>
         </is>
       </c>
       <c r="L14" s="9" t="inlineStr">
         <is>
-          <t>https://db.jobs/</t>
+          <t>https://apply.greateranglia.co.uk/</t>
         </is>
       </c>
       <c r="M14" s="12" t="inlineStr">
@@ -1859,85 +1867,153 @@
       </c>
       <c r="N14" s="7" t="inlineStr">
         <is>
-          <t>Search snippet</t>
+          <t>Old posting</t>
         </is>
       </c>
     </row>
     <row r="15" ht="110" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
+          <t>DB Cargo (freight)</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Junior Train Driver</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Not London-specific (national depots)</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>31381</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>55525</v>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>£31,381 start → £55,525 qualified.</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>~12–18 months</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Check advert</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>Depot dependent</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>Talent-pool style</t>
+        </is>
+      </c>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>https://db.jobs/</t>
+        </is>
+      </c>
+      <c r="M15" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>Search snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="110" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
           <t>GB Railfreight / Freightliner (freight)</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Trainee Train Driver</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Not London-specific</t>
         </is>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D16" s="8" t="n">
         <v>28937</v>
       </c>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>GBRf £28,937 training; qualified approx. £50–55k (GBRf), £50–56k (Freightliner) per industry summaries.</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>~12–18 months</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>Check advert</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I16" s="7" t="inlineStr">
         <is>
           <t>Not confirmed</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J16" s="7" t="inlineStr">
         <is>
           <t>Depot dependent</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr">
+      <c r="K16" s="7" t="inlineStr">
         <is>
           <t>Talent pool</t>
         </is>
       </c>
-      <c r="L15" s="9" t="inlineStr">
+      <c r="L16" s="9" t="inlineStr">
         <is>
           <t>https://careers.gbrailfreight.com/</t>
         </is>
       </c>
-      <c r="M15" s="12" t="inlineStr">
+      <c r="M16" s="12" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="N15" s="7" t="inlineStr">
+      <c r="N16" s="7" t="inlineStr">
         <is>
           <t>Industry summary figures</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>Confidence: High = official page read in full · Medium = official/advert detail via search · Low = forum, aggregator or dated source. Verify before applying.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N15"/>
+  <autoFilter ref="A1:N16"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -1953,6 +2029,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update train driver research with live careers-site checks via Chrome
Re-checked operators' job boards live on 4 Oct 2026: no London-area driver vacancies open; corrected Chiltern link; added Avanti official criteria.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/train_driver_research/london_train_driver_apprenticeships.xlsx
+++ b/train_driver_research/london_train_driver_apprenticeships.xlsx
@@ -853,7 +853,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Many operators' careers sites block automated access. Only Southeastern and LNER pages were read in full. Other rows come from job-advert snippets, press and forums, and some are 1–2 years old. See the 'Confidence' column (High / Medium / Low).</t>
+          <t>Salary figures for several operators still come from job-advert snippets, press and forums, some 1-2 years old - see the 'Confidence' column (High / Medium / Low). On 4 Oct 2026 the operators' own careers sites were re-checked live in Chrome (Southeastern, LNER, GTS/Elizabeth line, c2c, SWR, GTR, Chiltern, FirstGroup/GWR/First Rail London, EMR, Avanti, Greater Anglia, GB Railfreight, TfL apprenticeships) so vacancy status is current, but those sites mostly show no pay for roles that are not open.</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>4 Oct 2026 live check: the government Find an Apprenticeship service shows 0 train driver apprenticeships within 40 miles of London, and SWR and Elizabeth line (GTS) list no open driver vacancies – only talent pools. Several operators (TfL, East Midlands, London Northwestern, railforums) sit behind Cloudflare bot protection and could not be read; I did not try to bypass it.</t>
+          <t>4 Oct 2026 live check in Chrome: NONE of the London-area operators checked had a train driver vacancy open (Southeastern, GTS/Elizabeth line, c2c, SWR, GTR, Chiltern, GWR, First Rail London, EMR, LNER, Greater Anglia, GBRf); Avanti, GTS and SWR run register-interest talent pools. TfL's apprenticeships are closed, and TfL's job boards and DB Cargo (redirects to a German site) were not searched. Expect windows to open at short notice - register for alerts.</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>Closed 1 Jan 2026. Next window not announced – register for alerts</t>
+          <t>Closed 1 Jan 2026. Re-checked live in Chrome 4 Oct 2026: jobs.southeasternrailway.co.uk lists no driver roles (only Finance Business Partner, Railway Enforcement and Customer Service). Next window not announced - register for alerts</t>
         </is>
       </c>
       <c r="L2" s="9" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="N2" s="7" t="inlineStr">
         <is>
-          <t>Official advert read in full</t>
+          <t>Official advert read in full; live job board re-checked 4 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Closed 19 Jun 2026 (15 posts). Checked 4 Oct 2026: 0 driver vacancies, but a 'Trainee train driver' talent pool is open to register on careers.gtsr.co.uk</t>
+          <t>Closed 19 Jun 2026 (15 posts). Re-checked live in Chrome 4 Oct 2026: careers.gtsr.co.uk shows Drivers = 0 vacancies (only 1 Customer Experience role); register for job alerts</t>
         </is>
       </c>
       <c r="L3" s="9" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>TfL does not run a fixed cycle – posts on careers site when needed</t>
+          <t>No fixed cycle. Chrome check 4 Oct 2026: TfL careers page now loads; its Apprenticeships page says all roles are closed - register interest. TfL job boards sit behind a cookie wall and were not searched, so Tube driver (Train Operator) openings are unverified</t>
         </is>
       </c>
       <c r="L4" s="9" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="N4" s="7" t="inlineStr">
         <is>
-          <t>Forum figures; official TfL page blocked. Not confirmed as a formal Level 3 apprenticeship – ask TfL</t>
+          <t>Forum figures; official TfL careers/apprenticeships pages now read (no pay data or driver vacancy shown). Not confirmed as a formal Level 3 apprenticeship - ask TfL</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Check careers.c2c-online.co.uk</t>
+          <t>Checked live in Chrome 4 Oct 2026: only 2 vacancies (Business Continuity Manager, Quantity Surveyor), no driver roles - register interest on the site</t>
         </is>
       </c>
       <c r="L5" s="9" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>Aggregator advert snippet; official page had no live detail</t>
+          <t>Aggregator advert snippet for salary; official careers site read live 4 Oct 2026 (no driver roles, so salary cannot be confirmed)</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Checked 4 Oct 2026: no trainee driver vacancies listed – register for alerts</t>
+          <t>Checked live in Chrome 4 Oct 2026: job search shows 6 roles, none a driver. Homepage says talent pools for depots will open over the coming months - register for alerts</t>
         </is>
       </c>
       <c r="L6" s="9" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>Southern (Victoria) window opened Dec 2025 – check gtrailwaycareers.com for next</t>
+          <t>Southern (Victoria) window opened Dec 2025. Checked live in Chrome 4 Oct 2026: 9 vacancies, none a driver role - check gtrailwaycareers.com for next window</t>
         </is>
       </c>
       <c r="L7" s="9" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>Dated sources; careers site gave no live detail</t>
+          <t>Dated sources for pay; careers site read live 4 Oct 2026 (no driver vacancies)</t>
         </is>
       </c>
     </row>
@@ -1462,12 +1462,12 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>Talent pool opened Feb 2025 – check careers page</t>
+          <t>Talent pool opened Feb 2025. Checked live in Chrome 4 Oct 2026: Chiltern recruitment portal lists 11 jobs (first page), no driver roles seen</t>
         </is>
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>https://www.chilternrailways.co.uk/careers</t>
+          <t>https://ce0834li.webitrent.com/ce0834li_webrecruitment/wrd/run/ETREC179GF.open?WVID=68317141Hv</t>
         </is>
       </c>
       <c r="M8" s="11" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>Advert details via rail forum; consistent with other sources</t>
+          <t>Advert details via rail forum; consistent with other sources. Old /careers URL now 404s - link updated to the live recruitment portal</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>Rolling – via First Group careers</t>
+          <t>Checked live in Chrome 4 Oct 2026: FirstGroup job search has 0 vacancies in its Train Driver category (GWR roles open are dispatch/customer service/finance only)</t>
         </is>
       </c>
       <c r="L9" s="9" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Advertised 2026 – check careers page</t>
+          <t>Checked live in Chrome 4 Oct 2026: jobs.eastmidlandsrailway.co.uk lists no driver or apprentice roles (earlier 2026 advert has closed)</t>
         </is>
       </c>
       <c r="L10" s="9" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
-          <t>Search result summarising the live advert; official page blocked</t>
+          <t>Search result summarising an earlier advert; live EMR vacancy board read 4 Oct 2026 (no driver role open)</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1658,7 @@
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>None open at time of reading – register for job alerts</t>
+          <t>Checked live in Chrome 4 Oct 2026: apprenticeships page says no apprenticeship opportunities currently - register for job alerts</t>
         </is>
       </c>
       <c r="L11" s="9" t="inlineStr">
@@ -1673,7 +1673,7 @@
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>Official page read in full</t>
+          <t>Official page read in full; re-read live 4 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -1722,22 +1722,22 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Talent pool listed – register interest on Avanti careers site</t>
+          <t>No vacancy open. Avanti says to register interest and it will email when next recruiting trainee drivers (official page read in Chrome 4 Oct 2026). Official criteria: over 20.5 years old when applying, travel to depot within 1 hour, meet medical standards; circa £77,000 salary within a few years</t>
         </is>
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>https://www.avantiwestcoast.co.uk/careers</t>
+          <t>https://www.avantiwestcoast.co.uk/about-us/careers/train-driver-recruitment</t>
         </is>
       </c>
       <c r="M12" s="12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
-          <t>Aggregator listing only</t>
+          <t>Official Avanti train driver recruitment page read 4 Oct 2026 (age, depot radius, salary ceiling); no starting salary published</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>A window closed on a 23rd in May 2026 – details unconfirmed</t>
+          <t>No driver role open: FirstGroup job search 4 Oct 2026 shows 9 First Rail London roles, none train driver (Train Driver category = 0)</t>
         </is>
       </c>
       <c r="L13" s="9" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>Forum mention only</t>
+          <t>Forum mention for earlier window; live FirstGroup job board checked in Chrome 4 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>Currently advertising conductors (closed 7 Aug 2026) – drivers not confirmed</t>
+          <t>Checked live in Chrome 4 Oct 2026: "There are currently no positions advertised" on apply.greateranglia.co.uk - register interest</t>
         </is>
       </c>
       <c r="L14" s="9" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>Talent-pool style</t>
+          <t>Not checked - db.jobs redirects to the German DB site; check DB Cargo UK vacancies via the careers page</t>
         </is>
       </c>
       <c r="L15" s="9" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>Talent pool</t>
+          <t>Checked live in Chrome 4 Oct 2026: only Trainee Train Manager and Rail Operator talent pools (opening start of 2027) listed; no train driver role seen</t>
         </is>
       </c>
       <c r="L16" s="9" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="N16" s="7" t="inlineStr">
         <is>
-          <t>Industry summary figures</t>
+          <t>Industry summary figures; live GBRf careers site read 4 Oct 2026</t>
         </is>
       </c>
     </row>

</xml_diff>